<commit_message>
Format NT call/response examples like onboarding sample
Rewrite prerequisites 6–7 with Map.of + createInstance and
concrete HTTP/IT payloads matching ump-onboarding-pa style.

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-delete-documents-ncins-pa.xlsx
+++ b/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-delete-documents-ncins-pa.xlsx
@@ -881,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -902,7 +902,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs</t>
+          <t>UMP · п.6/п.7 в формате образца onboarding (Map.of)</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1">
+    <row r="6" ht="220" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>6</t>
@@ -958,19 +958,49 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Call Activity из main timeout (main BPMN в develop нет).
-Worker input (IT):
-{"businessKey":"550e8400-e29b-41d4-a716-446655110000","document":{"documentLink":"https://example.com/doc/123"}}</t>
+          <t xml:space="preserve">У воркера отсутствует HTTP-эндпоинт.
+Вызов происходит напрямую в Camunda.
+Camunda на базе Java скрипта, инструкция — https://confluence.moscow.alfaintra.net/pages/viewpage.action?pageId=2136656813
+Пример запроса:
+Map&lt;String, Object&gt; variables = Map.of(
+  "businessKey", "550e8400-e29b-41d4-a716-446655110003", // id заявки (UMP application)
+  "productCode", "NON_CREDIT_INSURANCE" // const
+);
+final ProcessInstanceEvent processInstanceEvent = client
+  .newCreateInstanceCommand()
+  .bpmnProcessId("ump-delete-documents-ncins-pa")
+  .latestVersion()
+  .variables(variables)
+  .send()
+  .join();
+Параметры для запроса:
+1. businessKey — UUID заявки (параметризовать на объём ≥ ЧПН)
+2. productCode — const NON_CREDIT_INSURANCE (параметризация не нужна)
+Обычно стартует Call Activity из main timeout (не напрямую).
+--- Шаги (DeleteDocumentsWorkerIT) ---
+1) get-application-data processType=DELETE_DOCS
+Map.of("businessKey", "550e8400-e29b-41d4-a716-446655110000", "processType", "DELETE_DOCS");
+HTTP: GET .../applications/550e8400-e29b-41d4-a716-446655110000?include=PARTICIPANT&amp;include=PRODUCT
+→ documents = [{"documentLink": "&lt;contract|policy|agreement link&gt;"}]
+2) delete-documents (multiInstance, каждый document)
+Map.of(
+  "businessKey", "550e8400-e29b-41d4-a716-446655110000",
+  "document", "{ "documentLink": "https://example.com/doc/123" }"
+);
+HTTP: отсутствует (DeleteDocumentsService TODO AC 1.0 stub)
+</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>DeleteDocumentsWorkerIT</t>
+          <t>Map.of start/Call Activity + stub delete</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Сначала нужно добыть живой пример вызова сервиса (локально/стенд) и параметризовать.</t>
+          <t>Сначала нужно добыть живой пример вызова сервиса (локально/стенд) и параметризовать.
+Параметризовать businessKey (≥ ЧПН). productCode — const NON_CREDIT_INSURANCE.
+Источник примеров: develop ump-ncins-pa *WorkerIT + stubs.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -979,7 +1009,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="70" customHeight="1">
+    <row r="7" ht="180" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>7</t>
@@ -992,9 +1022,13 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Success: {"documentResponse":{"status":"1"}}
-Exception path: status="2".
-Реальный AC deleteDocsh — TBD (TODO в DeleteDocumentsService).</t>
+          <t>Camunda out (IT):
+{ "documentResponse": { "status": "1" } }
+При exception в сервисе:
+{ "documentResponse": { "status": "2" } }
+get-application-data: getProcessParams = SUCCESS | ERROR
+Реальный AC deleteDocsh request/response — TBD после снятия stub
+(как в образце п.7: если нет — прогнать локально/стенд и сохранить ответ).</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1004,7 +1038,9 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Нужны примеры ответов, которые можно считать ожидаемыми.</t>
+          <t>Нужны примеры ответов, которые можно считать ожидаемыми.
+Например: getProcessParams=SUCCESS; HTTP 200/201; result=SUCCESS.
+Источник: *WorkerIT + stubs/ump/ump_application_response_200.json.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -1175,6 +1211,14 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add full HTTP request/response bodies to NT method sheets
Replace short method names with complete headers and JSON
bodies from WorkerIT stubs (applications, ins-contracts, etc.).

Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-delete-documents-ncins-pa.xlsx
+++ b/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-delete-documents-ncins-pa.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +52,10 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -93,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,6 +110,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -494,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs</t>
+          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs · полные HTTP body</t>
         </is>
       </c>
     </row>
@@ -565,7 +572,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs</t>
+          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs · полные HTTP body</t>
         </is>
       </c>
     </row>
@@ -632,7 +639,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs</t>
+          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs · полные HTTP body</t>
         </is>
       </c>
     </row>
@@ -881,7 +888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -902,7 +909,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · п.6/п.7 в формате образца onboarding (Map.of)</t>
+          <t>UMP · п.6/п.7 в формате образца onboarding (Map.of) · полные HTTP body</t>
         </is>
       </c>
     </row>
@@ -1211,14 +1218,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1234,11 +1233,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1251,14 +1250,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>UMP · 21 июля 2026 · код develop ump-ncins-pa@4a921a1653e + IT stubs</t>
+          <t>Полные request/response (не только имя метода). Источник: develop ump-ncins-pa@4a921a1653e + *WorkerIT + stubs. · полные HTTP body</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Методы delete (develop + IT)</t>
+          <t>HTTP / JobWorker — полные тела запросов и ответов</t>
         </is>
       </c>
     </row>
@@ -1270,91 +1269,257 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>BPMN / JobWorker</t>
+          <t>Метод / JobWorker</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Где</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Type / HTTP</t>
+          <t>Полный REQUEST (headers + body)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Request / Input</t>
+          <t>Полный RESPONSE (status + body)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Response / Output</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+          <t>Источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="420" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>get-application-data</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>ApplicationDataWorker</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>GET /applications/{id}</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>processType=DELETE_DOCS</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>documents[{documentLink}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>ump-delete-documents-ncins-pa.delete-documents</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>DeleteDocumentsWorker</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>STUB (TODO AC 1.0)</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>document.documentLink</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>{"documentResponse":{"status":"1"}}</t>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>get-application-data
+GET /applications/{id}</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>ApplicationDataWorker
+все процессы</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>GET /applications/6dc5daf3-da12-4aae-9766-572da7b6b003?include=PARTICIPANT&amp;include=PRODUCT HTTP/1.1
+Host: ump-application-facade.ump.svc.cluster.local
+Accept: application/json
+(без body)
+Camunda job input:
+{
+  "businessKey": "6dc5daf3-da12-4aae-9766-572da7b6b003",
+  "processType": "&lt;PREPARE_DOCUMENTS|SIGNING|PAYMENT|FINALISATION|DELETE_DOCS&gt;"
+}</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>HTTP/1.1 200 OK
+Content-Type: application/json
+{
+  "externalApplicationIds": [
+    {
+      "extAppId": "7ca85f64-5717-4562-b3fc-6c163f65aba9",
+      "systemCode": "SFA",
+      "extAppCreateDate": "2026-06-25T12:45:34.785179Z"
+    }
+  ],
+  "channels": [
+    {
+      "id": "bd458000-77c2-48af-91b4-815f7ef2d4e6",
+      "userInfo": {
+        "userId": "f6753df0-b5c9-4828-a7b7-f9f3f7d8f33c",
+        "login": "service-account-nib-corp-ncins"
+      },
+      "code": "nib-corp-ncins",
+      "name": "НИБ. Страхование",
+      "isDeleted": false,
+      "category": "RECEIVE",
+      "type": "BANK_SYSTEM"
+    }
+  ],
+  "participants": [
+    {
+      "id": "bdec62a5-e10a-4c5b-86c7-b5ac190b8055",
+      "applicationId": "6dc5daf3-da12-4aae-9766-572da7b6b003",
+      "isDeleted": false,
+      "contacts": [
+        {
+          "type": "EMAIL",
+          "typeName": "Email",
+          "value": "romashka@rambler.ru",
+          "isPrimary": false
+        },
+        {
+          "type": "PHONE",
+          "typeName": "Телефон",
+          "value": "79183221488",
+          "isPrimary": false
+        }
+      ],
+      "addresses": [
+        {
+          "type": "FACT",
+          "typeName": "Адрес проживания / фактический - краткий",
+          "address": {
+            "fullAddress": "Г. Пушкино ул. Колотушкина д. 14/88"
+          }
+        }
+      ],
+      "identityDocuments": [],
+      "okveds": [],
+      "licenses": [],
+      "management": [],
+      "founders": [],
+      "externalPins": [],
+      "pin": "AAAXYX",
+      "type": "LEGAL",
+      "typeName": "Юридическое лицо",
+      "fullName": "ООО Звезда",
+      "inn": "7826688577",
+      "createDate": "2026-07-09T17:19:18.963685Z",
+      "lastUpdateDate": "2026-07-09T17:19:19.99786Z",
+      "citizenship": "Россия",
+      "citizenshipCode": "RU",
+      "taxCountryCode": "RU",
+      "ogrn": "1027810281740"
+    }
+  ],
+  "products": [
+    {
+      "id": "3d9fe175-2bc5-442a-b900-48522551de3f",
+      "applicationId": "6dc5daf3-da12-4aae-9766-572da7b6b003",
+      "status": {
+        "isTerminate": true,
+        "code": "COMPLETE",
+        "name": "Завершен"
+      },
+      "stage": {
+        "code": "PAYMENT_COMPLETED",
+        "name": "PAYMENT_COMPLETED"
+      },
+      "createDate": "2026-07-09T17:19:18.891861Z",
+      "lastUpdateDate": "2026-07-09T17:23:50.600316Z",
+      "code": "NON_CREDIT_INSURANCE",
+      "name": "Некредитное страхование ЮЛ",
+      "type": "PRODUCT",
+      "main": false,
+      "isDeleted": false,
+      "responsibleManager": {
+        "login": "U_M13RU"
+      },
+      "salesChannel": {
+        "code": "SFA",
+        "name": "SFA"
+      },
+      "productProperties": {
+        "programId": 1073741824,
+        "beginDate": "2026-06-25T11:47:13.57Z",
+        "endDate": "2026-06-25T11:47:13.57Z",
+        "signDate": "2026-06-25T11:47:13.57Z",
+        "duration": 12,
+        "insuranceSum": 20000.0,
+        "insurancePremium": 20000.0,
+        "contractNumber": "1423423/sdf/123",
+        "paymentType": "payment_account",
+        "agreementLink": "7ca85f64-5717-4562-b3fc-6c163f65aba9",
+        "insuranceObjects": [
+          {
+            "paymentAccount": "123523464567347"
+          }
+        ],
+        "code": "NON_CREDIT_INSURANCE"
+      },
+      "channelCode": "nib-corp-ncins"
+    }
+  ],
+  "options": [],
+  "id": "6dc5daf3-da12-4aae-9766-572da7b6b003",
+  "createDate": "2026-07-09T17:19:18.833504Z",
+  "lastUpdateDate": "2026-07-09T17:22:46.462517Z",
+  "number": "UMP26070994592",
+  "statusCode": "COMPLETE",
+  "statusName": "Завершена",
+  "finalVersion": true,
+  "isDeleted": false
+}
+Camunda job output (успех):
+{ "getProcessParams": "SUCCESS", ...поля по processType из ApplicationMapper }
+Ошибка:
+{ "getProcessParams": "ERROR" }</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>ApplicationDataWorkerIT
+stubs/ump/ump_application_response_200.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="204" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>ump-delete-documents-ncins-pa.delete-documents
+STUB AC 1.0</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>DeleteDocumentsWorker
+delete</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>JobWorker: ump-delete-documents-ncins-pa.delete-documents
+HTTP: нет (DeleteDocumentsService TODO AC 1.0 stub)
+Camunda input (DeleteDocumentsWorkerIT / multiInstance element):
+{
+  "businessKey": "550e8400-e29b-41d4-a716-446655110000",
+  "document": {
+    "documentLink": "https://example.com/doc/123"
+  }
+}</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Camunda output:
+{
+  "documentResponse": {
+    "status": "1"
+  }
+}
+При exception:
+{
+  "documentResponse": {
+    "status": "2"
+  }
+}
+Реальный POST AlfaCapture deleteDocsh — TBD (stub).</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>DeleteDocumentsWorkerIT
+DeleteDocumentsService stub</t>
         </is>
       </c>
     </row>

</xml_diff>